<commit_message>
Update registrations sheet and package lock
</commit_message>
<xml_diff>
--- a/exports/registrations.xlsx
+++ b/exports/registrations.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U77"/>
+  <dimension ref="A1:U83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8"/>
@@ -7478,12 +7478,618 @@
       </c>
       <c r="T77" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="U77" t="inlineStr">
         <is>
           <t>02-06-2026 05:55 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>69</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>REG-45D503F3</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>L - 9545</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Test Devotee 9545</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>30</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>9441669545</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q78" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>TXN9545</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>70</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>REG-5A3FC903</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>L - 98765</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Traceback Finder</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>40</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>9441665181</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q79" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>TXN9876543210</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:46 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>71</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>REG-6495C520</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>L - 11111</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>File Upload Tester</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>25</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>9441665181</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q80" t="n">
+        <v>1800</v>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>TXN1111111111</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:50 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>72</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>REG-22C57439</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>L - 893164</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Random Devotee 893164</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>28</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>9876893164</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Non-Kriyaban</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q81" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>TXN893164</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>11-06-2026 07:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>73</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>REG-A14952A9</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>NEW MEMBER 7</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Test Browser Subagent</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>28</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>9111122222</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>browser_test@example.com</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Non-Kriyaban</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q82" t="n">
+        <v>1800</v>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>TXN_BROWSER_123</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>11-06-2026 08:17 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>74</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>REG-5B375D48</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>NEW MEMBER 8</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Local Browser Test 5001</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>29</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>local_test@example.com</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q83" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>TXN_LOCAL_5001</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>11-06-2026 08:28 AM</t>
         </is>
       </c>
     </row>
@@ -7498,12 +8104,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U45"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="5" customWidth="1" min="6" max="6"/>
@@ -12075,6 +12681,410 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>REG-45D503F3</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>L - 9545</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Test Devotee 9545</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>30</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>9441669545</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>TXN9545</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>REG-5A3FC903</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>L - 98765</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Traceback Finder</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>40</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>9441665181</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>TXN9876543210</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:46 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>REG-6495C520</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>L - 11111</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>File Upload Tester</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>25</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>9441665181</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>1800</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>TXN1111111111</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:50 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>REG-5B375D48</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NEW MEMBER 8</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Local Browser Test 5001</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>29</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>local_test@example.com</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>TXN_LOCAL_5001</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>11-06-2026 08:28 AM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12086,7 +13096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14634,12 +15644,214 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
           <t>02-06-2026 05:55 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>REG-22C57439</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>L - 893164</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Random Devotee 893164</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>28</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9876893164</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Non-Kriyaban</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>TXN893164</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>11-06-2026 07:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>REG-A14952A9</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>NEW MEMBER 7</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Test Browser Subagent</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>28</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>9111122222</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>browser_test@example.com</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Non-Kriyaban</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>1800</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>TXN_BROWSER_123</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>11-06-2026 08:17 AM</t>
         </is>
       </c>
     </row>
@@ -14654,7 +15866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16908,6 +18120,410 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>REG-45D503F3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>L - 9545</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Test Devotee 9545</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>30</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>9441669545</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>TXN9545</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>REG-5A3FC903</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>L - 98765</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Traceback Finder</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>40</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>9441665181</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>TXN9876543210</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>11-06-2026 04:46 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>REG-22C57439</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>L - 893164</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Random Devotee 893164</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>9876893164</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>anantapur@ysscenters.org</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Non-Kriyaban</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>TXN893164</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>11-06-2026 07:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>REG-5B375D48</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>NEW MEMBER 8</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Local Browser Test 5001</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>29</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>local_test@example.com</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Kriyaban</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>2800</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>TXN_LOCAL_5001</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>11-06-2026 08:28 AM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>